<commit_message>
Improve ERP workflows and interface
</commit_message>
<xml_diff>
--- a/apps/admin/public/templates/采购申请批量导入模板.xlsx
+++ b/apps/admin/public/templates/采购申请批量导入模板.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购明细" sheetId="1" r:id="R0e6396b535e040d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R83973cc848124d06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采购明细" sheetId="1" r:id="Ra5662a0cd6ce46d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rdccfd11c6cb649c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -420,7 +420,7 @@
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
@@ -462,7 +462,7 @@
         <x:v>数量*</x:v>
       </x:c>
       <x:c r="D4" s="14" t="str">
-        <x:v>预计单价</x:v>
+        <x:v>预计单价（含税，元）</x:v>
       </x:c>
       <x:c r="E4" s="14" t="str">
         <x:v>税率(%)</x:v>
@@ -1502,7 +1502,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
@@ -1574,7 +1574,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="25" t="str">
-        <x:v>预计单价</x:v>
+        <x:v>预计单价（含税，元）</x:v>
       </x:c>
       <x:c r="B7" s="28" t="str">
         <x:v>否</x:v>

</xml_diff>